<commit_message>
MERCADO NPH: excluir pisos 2 y 3 (ofertas 1 y 3) y enlace directo oferta 2
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X48yXL1Fu4ZbLk5QBNEV96
</commit_message>
<xml_diff>
--- a/ESTUDIO_MERCADO_URBANO_BELLO_NPH_depurado.xlsx
+++ b/ESTUDIO_MERCADO_URBANO_BELLO_NPH_depurado.xlsx
@@ -1409,7 +1409,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="es-CO"/>
               </a:p>
@@ -1647,7 +1647,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="es-CO"/>
           </a:p>
@@ -1738,7 +1738,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="es-CO"/>
           </a:p>
@@ -1849,7 +1849,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="es-CO"/>
               </a:p>
@@ -2065,7 +2065,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="es-CO"/>
           </a:p>
@@ -2156,7 +2156,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="es-CO"/>
           </a:p>
@@ -32477,12 +32477,12 @@
       </c>
       <c r="Y9" s="94" t="inlineStr">
         <is>
-          <t>Casa urbana ≤100 m² en Niquía con lote declarado; falta edad y estado.</t>
+          <t>NO – segundo piso (dúplex), derecho sobre un piso; enlace pendiente de verificar (Ciencuadras 3374259). Casa urbana ≤100 m² en Niquía con lote declarado; falta edad y estado.</t>
         </is>
       </c>
       <c r="Z9" s="94" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AA9" s="191">
@@ -32593,7 +32593,7 @@
       </c>
       <c r="X10" s="100" t="inlineStr">
         <is>
-          <t>https://www.fincaraiz.com.co/venta/altos-de-niquia/bello</t>
+          <t>https://www.fincaraiz.com.co/casa-en-venta-en-bello/192592199</t>
         </is>
       </c>
       <c r="Y10" s="94" t="inlineStr">
@@ -32721,12 +32721,12 @@
       </c>
       <c r="Y11" s="94" t="inlineStr">
         <is>
-          <t>Derechos sobre un piso; área total 140 m² supera el máximo de 100 m².</t>
+          <t>NO – tercer piso; fuera del estudio de NPH. Derechos sobre un piso; área total 140 m² supera el máximo de 100 m².</t>
         </is>
       </c>
       <c r="Z11" s="94" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="AA11" s="191">
@@ -35335,6 +35335,9 @@
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
MERCADO NPH: ingresar 5 ofertas nuevas (filas 23-27) de Doomos y MercadoLibre
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X48yXL1Fu4ZbLk5QBNEV96
</commit_message>
<xml_diff>
--- a/ESTUDIO_MERCADO_URBANO_BELLO_NPH_depurado.xlsx
+++ b/ESTUDIO_MERCADO_URBANO_BELLO_NPH_depurado.xlsx
@@ -34084,21 +34084,56 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="103" t="n"/>
-      <c r="B23" s="93" t="n"/>
-      <c r="C23" s="94" t="n"/>
-      <c r="D23" s="94" t="n"/>
-      <c r="E23" s="94" t="n"/>
-      <c r="F23" s="94" t="n"/>
-      <c r="G23" s="94" t="n"/>
-      <c r="H23" s="94" t="n"/>
-      <c r="I23" s="189" t="n"/>
-      <c r="J23" s="190" t="n"/>
+      <c r="A23" s="103" t="n">
+        <v>15</v>
+      </c>
+      <c r="B23" s="93" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C23" s="94" t="inlineStr">
+        <is>
+          <t>Casa-lote</t>
+        </is>
+      </c>
+      <c r="D23" s="94" t="inlineStr">
+        <is>
+          <t>Oferta de venta</t>
+        </is>
+      </c>
+      <c r="E23" s="94" t="inlineStr">
+        <is>
+          <t>Bello</t>
+        </is>
+      </c>
+      <c r="F23" s="94" t="inlineStr">
+        <is>
+          <t>Niquía Camacol (parte baja)</t>
+        </is>
+      </c>
+      <c r="G23" s="94" t="inlineStr">
+        <is>
+          <t>Niquía Camacol parte baja, Bello</t>
+        </is>
+      </c>
+      <c r="H23" s="94" t="inlineStr">
+        <is>
+          <t>6.342933, -75.551884</t>
+        </is>
+      </c>
+      <c r="I23" s="189" t="n">
+        <v>380000000</v>
+      </c>
+      <c r="J23" s="190">
+        <f>DATOS!$C$17</f>
+        <v/>
+      </c>
       <c r="K23" s="191">
         <f>IF(I23="","",I23*(1-J23))</f>
         <v/>
       </c>
-      <c r="L23" s="98" t="n"/>
+      <c r="L23" s="98" t="n">
+        <v>216</v>
+      </c>
       <c r="M23" s="98" t="n"/>
       <c r="N23" s="192">
         <f>IF(A23="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A23))</f>
@@ -34120,14 +34155,42 @@
         <f>IF(OR(K23="",N(M23)&lt;=0),"",K23/M23)</f>
         <v/>
       </c>
-      <c r="S23" s="94" t="n"/>
+      <c r="S23" s="94" t="inlineStr">
+        <is>
+          <t>Por verificar en POT de Bello (Acuerdo vigente)</t>
+        </is>
+      </c>
       <c r="T23" s="94" t="n"/>
-      <c r="U23" s="94" t="n"/>
-      <c r="V23" s="94" t="n"/>
-      <c r="W23" s="94" t="n"/>
-      <c r="X23" s="102" t="n"/>
-      <c r="Y23" s="94" t="n"/>
-      <c r="Z23" s="94" t="n"/>
+      <c r="U23" s="94" t="inlineStr">
+        <is>
+          <t>Lote con casa para remodelar (ladrillo, piso en cemento), 2 alcobas, 1 baño, cocina sencilla sin gas. Cód. 6662. Ficha Doomos: 30/08/2026 y "2 días en el mercado · actualizado hoy" (fecha inconsistente). No publica piso, régimen ni administración ni área construida.</t>
+        </is>
+      </c>
+      <c r="V23" s="94" t="inlineStr">
+        <is>
+          <t>La Palma Inmobiliaria S.A.S. – Doomos</t>
+        </is>
+      </c>
+      <c r="W23" s="94" t="inlineStr">
+        <is>
+          <t>Solicitar en portal</t>
+        </is>
+      </c>
+      <c r="X23" s="102" t="inlineStr">
+        <is>
+          <t>https://www.doomos.com.co/propiedad/lote-casa-en-venta-en-bello-cod-6662</t>
+        </is>
+      </c>
+      <c r="Y23" s="94" t="inlineStr">
+        <is>
+          <t>Casa-lote 216 m² (fuera del rango 80–120 m²); incluida por decisión del perito. Falta área construida, nivel y régimen.</t>
+        </is>
+      </c>
+      <c r="Z23" s="94" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AA23" s="191">
         <f>IF(AND(Z23="SÍ",ISNUMBER(R23)),R23,"")</f>
         <v/>
@@ -34146,21 +34209,52 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="92" t="n"/>
-      <c r="B24" s="93" t="n"/>
-      <c r="C24" s="94" t="n"/>
-      <c r="D24" s="94" t="n"/>
-      <c r="E24" s="94" t="n"/>
-      <c r="F24" s="94" t="n"/>
-      <c r="G24" s="94" t="n"/>
+      <c r="A24" s="92" t="n">
+        <v>16</v>
+      </c>
+      <c r="B24" s="93" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C24" s="94" t="inlineStr">
+        <is>
+          <t>Casa-lote</t>
+        </is>
+      </c>
+      <c r="D24" s="94" t="inlineStr">
+        <is>
+          <t>Oferta de venta</t>
+        </is>
+      </c>
+      <c r="E24" s="94" t="inlineStr">
+        <is>
+          <t>Bello</t>
+        </is>
+      </c>
+      <c r="F24" s="94" t="inlineStr">
+        <is>
+          <t>Niquía</t>
+        </is>
+      </c>
+      <c r="G24" s="94" t="inlineStr">
+        <is>
+          <t>Niquía, Bello, Antioquia</t>
+        </is>
+      </c>
       <c r="H24" s="94" t="n"/>
-      <c r="I24" s="189" t="n"/>
-      <c r="J24" s="190" t="n"/>
+      <c r="I24" s="189" t="n">
+        <v>600000000</v>
+      </c>
+      <c r="J24" s="190">
+        <f>DATOS!$C$17</f>
+        <v/>
+      </c>
       <c r="K24" s="191">
         <f>IF(I24="","",I24*(1-J24))</f>
         <v/>
       </c>
-      <c r="L24" s="98" t="n"/>
+      <c r="L24" s="98" t="n">
+        <v>129</v>
+      </c>
       <c r="M24" s="98" t="n"/>
       <c r="N24" s="192">
         <f>IF(A24="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A24))</f>
@@ -34182,14 +34276,42 @@
         <f>IF(OR(K24="",N(M24)&lt;=0),"",K24/M24)</f>
         <v/>
       </c>
-      <c r="S24" s="94" t="n"/>
+      <c r="S24" s="94" t="inlineStr">
+        <is>
+          <t>Por verificar en POT de Bello (Acuerdo vigente)</t>
+        </is>
+      </c>
       <c r="T24" s="94" t="n"/>
-      <c r="U24" s="94" t="n"/>
-      <c r="V24" s="94" t="n"/>
-      <c r="W24" s="94" t="n"/>
-      <c r="X24" s="102" t="n"/>
-      <c r="Y24" s="94" t="n"/>
-      <c r="Z24" s="94" t="n"/>
+      <c r="U24" s="94" t="inlineStr">
+        <is>
+          <t>Casa de primer piso para remodelar, 4 habitaciones, 1 baño, sala, comedor, cocina integral, cuarto útil; 129 m² totales (no separa lote de construcción). Cerca al colegio Consejo de Bello. No publica régimen, administración ni coordenadas.</t>
+        </is>
+      </c>
+      <c r="V24" s="94" t="inlineStr">
+        <is>
+          <t>Myeinmobiliariasas – MercadoLibre</t>
+        </is>
+      </c>
+      <c r="W24" s="94" t="inlineStr">
+        <is>
+          <t>Solicitar en portal</t>
+        </is>
+      </c>
+      <c r="X24" s="102" t="inlineStr">
+        <is>
+          <t>https://casa.mercadolibre.com.co/MCO-2237453771-casa-lote-en-venta-niquia-bello-_JM</t>
+        </is>
+      </c>
+      <c r="Y24" s="94" t="inlineStr">
+        <is>
+          <t>Casa-lote primer piso; 129 m² totales sin separar lote/construido. Falta confirmar régimen, administración y coordenadas.</t>
+        </is>
+      </c>
+      <c r="Z24" s="94" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AA24" s="191">
         <f>IF(AND(Z24="SÍ",ISNUMBER(R24)),R24,"")</f>
         <v/>
@@ -34208,21 +34330,52 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="81" t="n"/>
-      <c r="B25" s="82" t="n"/>
-      <c r="C25" s="83" t="n"/>
-      <c r="D25" s="83" t="n"/>
-      <c r="E25" s="83" t="n"/>
-      <c r="F25" s="83" t="n"/>
-      <c r="G25" s="83" t="n"/>
+      <c r="A25" s="81" t="n">
+        <v>17</v>
+      </c>
+      <c r="B25" s="82" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C25" s="83" t="inlineStr">
+        <is>
+          <t>Casa-lote</t>
+        </is>
+      </c>
+      <c r="D25" s="83" t="inlineStr">
+        <is>
+          <t>Oferta de venta</t>
+        </is>
+      </c>
+      <c r="E25" s="83" t="inlineStr">
+        <is>
+          <t>Bello</t>
+        </is>
+      </c>
+      <c r="F25" s="83" t="inlineStr">
+        <is>
+          <t>Barrio Nuevo</t>
+        </is>
+      </c>
+      <c r="G25" s="83" t="inlineStr">
+        <is>
+          <t>Barrio Nuevo, Bello, Antioquia</t>
+        </is>
+      </c>
       <c r="H25" s="83" t="n"/>
-      <c r="I25" s="193" t="n"/>
-      <c r="J25" s="194" t="n"/>
+      <c r="I25" s="193" t="n">
+        <v>495000000</v>
+      </c>
+      <c r="J25" s="194">
+        <f>DATOS!$C$17</f>
+        <v/>
+      </c>
       <c r="K25" s="195">
         <f>IF(I25="","",I25*(1-J25))</f>
         <v/>
       </c>
-      <c r="L25" s="87" t="n"/>
+      <c r="L25" s="87" t="n">
+        <v>120</v>
+      </c>
       <c r="M25" s="87" t="n"/>
       <c r="N25" s="196">
         <f>IF(A25="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A25))</f>
@@ -34244,14 +34397,42 @@
         <f>IF(OR(K25="",N(M25)&lt;=0),"",K25/M25)</f>
         <v/>
       </c>
-      <c r="S25" s="83" t="n"/>
+      <c r="S25" s="83" t="inlineStr">
+        <is>
+          <t>Por verificar en POT de Bello (Acuerdo vigente)</t>
+        </is>
+      </c>
       <c r="T25" s="83" t="n"/>
-      <c r="U25" s="83" t="n"/>
-      <c r="V25" s="83" t="n"/>
-      <c r="W25" s="83" t="n"/>
-      <c r="X25" s="89" t="n"/>
-      <c r="Y25" s="83" t="n"/>
-      <c r="Z25" s="83" t="n"/>
+      <c r="U25" s="83" t="inlineStr">
+        <is>
+          <t>Casa unifamiliar con aire, 4 habitaciones, 2 baños, 2 patios, sala-comedor, cocina semiintegral; 120 m² totales (no separa lote/construido). Publicada hace 9 días (a 05/10/2026). No publica nivel, régimen, administración ni coordenadas.</t>
+        </is>
+      </c>
+      <c r="V25" s="83" t="inlineStr">
+        <is>
+          <t>Myeinmobiliariasas – MercadoLibre</t>
+        </is>
+      </c>
+      <c r="W25" s="83" t="inlineStr">
+        <is>
+          <t>Solicitar en portal</t>
+        </is>
+      </c>
+      <c r="X25" s="89" t="inlineStr">
+        <is>
+          <t>https://casa.mercadolibre.com.co/MCO-2237592443-casa-lote-en-venta-en-barrio-nuevo-bello-_JM</t>
+        </is>
+      </c>
+      <c r="Y25" s="83" t="inlineStr">
+        <is>
+          <t>Casa-lote 120 m² totales sin separar lote/construido. Falta nivel, régimen, administración y coordenadas; barrio por confirmar distancia al objeto.</t>
+        </is>
+      </c>
+      <c r="Z25" s="83" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AA25" s="195">
         <f>IF(AND(Z25="SÍ",ISNUMBER(R25)),R25,"")</f>
         <v/>
@@ -34270,21 +34451,52 @@
       </c>
     </row>
     <row r="26" hidden="1" s="54">
-      <c r="A26" s="70" t="n"/>
-      <c r="B26" s="71" t="n"/>
-      <c r="C26" s="70" t="n"/>
-      <c r="D26" s="70" t="n"/>
-      <c r="E26" s="70" t="n"/>
-      <c r="F26" s="70" t="n"/>
-      <c r="G26" s="70" t="n"/>
+      <c r="A26" s="70" t="n">
+        <v>18</v>
+      </c>
+      <c r="B26" s="71" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C26" s="70" t="inlineStr">
+        <is>
+          <t>Casa-lote</t>
+        </is>
+      </c>
+      <c r="D26" s="70" t="inlineStr">
+        <is>
+          <t>Oferta de venta</t>
+        </is>
+      </c>
+      <c r="E26" s="70" t="inlineStr">
+        <is>
+          <t>Bello</t>
+        </is>
+      </c>
+      <c r="F26" s="70" t="inlineStr">
+        <is>
+          <t>Mesa</t>
+        </is>
+      </c>
+      <c r="G26" s="70" t="inlineStr">
+        <is>
+          <t>Barrio Mesa, a una cuadra de la Obra 2000, contiguo a fruver, Bello</t>
+        </is>
+      </c>
       <c r="H26" s="70" t="n"/>
-      <c r="I26" s="197" t="n"/>
-      <c r="J26" s="198" t="n"/>
+      <c r="I26" s="197" t="n">
+        <v>390000000</v>
+      </c>
+      <c r="J26" s="198">
+        <f>DATOS!$C$17</f>
+        <v/>
+      </c>
       <c r="K26" s="199">
         <f>IF(I26="","",I26*(1-J26))</f>
         <v/>
       </c>
-      <c r="L26" s="73" t="n"/>
+      <c r="L26" s="73" t="n">
+        <v>120</v>
+      </c>
       <c r="M26" s="73" t="n"/>
       <c r="N26" s="200">
         <f>IF(A26="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A26))</f>
@@ -34306,14 +34518,42 @@
         <f>IF(OR(K26="",N(M26)&lt;=0),"",K26/M26)</f>
         <v/>
       </c>
-      <c r="S26" s="70" t="n"/>
+      <c r="S26" s="70" t="inlineStr">
+        <is>
+          <t>Por verificar en POT de Bello (Acuerdo vigente)</t>
+        </is>
+      </c>
       <c r="T26" s="70" t="n"/>
-      <c r="U26" s="70" t="n"/>
-      <c r="V26" s="70" t="n"/>
-      <c r="W26" s="70" t="n"/>
-      <c r="X26" s="70" t="n"/>
-      <c r="Y26" s="70" t="n"/>
-      <c r="Z26" s="74" t="n"/>
+      <c r="U26" s="70" t="inlineStr">
+        <is>
+          <t>Casa-lote apta para construir apartamentos o locales. Escritura: 8 x 18 m; real aproximadamente 120 m². Ficha: 120 m² totales. Publicada hace 5 días (a 05/10/2026). No publica nivel, régimen, administración ni coordenadas.</t>
+        </is>
+      </c>
+      <c r="V26" s="70" t="inlineStr">
+        <is>
+          <t>Aviarrendamientosvicasas – MercadoLibre</t>
+        </is>
+      </c>
+      <c r="W26" s="70" t="inlineStr">
+        <is>
+          <t>Solicitar en portal</t>
+        </is>
+      </c>
+      <c r="X26" s="70" t="inlineStr">
+        <is>
+          <t>https://casa.mercadolibre.com.co/MCO-4493777078-vendo-casa-lote-obra-2000-barrio-mesa-bello-_JM</t>
+        </is>
+      </c>
+      <c r="Y26" s="70" t="inlineStr">
+        <is>
+          <t>Casa-lote ~120 m² reales (escritura 144 m²). Falta nivel, régimen, administración y coordenadas.</t>
+        </is>
+      </c>
+      <c r="Z26" s="74" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AA26" s="199">
         <f>IF(AND(Z26="SÍ",ISNUMBER(R26)),R26,"")</f>
         <v/>
@@ -34332,22 +34572,53 @@
       </c>
     </row>
     <row r="27" hidden="1" s="54">
-      <c r="A27" s="70" t="n"/>
-      <c r="B27" s="71" t="n"/>
-      <c r="C27" s="70" t="n"/>
-      <c r="D27" s="70" t="n"/>
-      <c r="E27" s="70" t="n"/>
-      <c r="F27" s="70" t="n"/>
-      <c r="G27" s="70" t="n"/>
+      <c r="A27" s="70" t="n">
+        <v>19</v>
+      </c>
+      <c r="B27" s="71" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C27" s="70" t="inlineStr">
+        <is>
+          <t>Casa</t>
+        </is>
+      </c>
+      <c r="D27" s="70" t="inlineStr">
+        <is>
+          <t>Oferta de venta</t>
+        </is>
+      </c>
+      <c r="E27" s="70" t="inlineStr">
+        <is>
+          <t>Bello</t>
+        </is>
+      </c>
+      <c r="F27" s="70" t="inlineStr">
+        <is>
+          <t>Santa Ana</t>
+        </is>
+      </c>
+      <c r="G27" s="70" t="inlineStr">
+        <is>
+          <t>Santa Ana, cerca a La Salle Super Punto, Bello</t>
+        </is>
+      </c>
       <c r="H27" s="70" t="n"/>
-      <c r="I27" s="197" t="n"/>
-      <c r="J27" s="198" t="n"/>
+      <c r="I27" s="197" t="n">
+        <v>390000000</v>
+      </c>
+      <c r="J27" s="198">
+        <f>DATOS!$C$17</f>
+        <v/>
+      </c>
       <c r="K27" s="199">
         <f>IF(I27="","",I27*(1-J27))</f>
         <v/>
       </c>
       <c r="L27" s="73" t="n"/>
-      <c r="M27" s="73" t="n"/>
+      <c r="M27" s="73" t="n">
+        <v>168</v>
+      </c>
       <c r="N27" s="200">
         <f>IF(A27="","",SUMIFS(DEPRECIACIÓN!$P$5:$P$24,DEPRECIACIÓN!$A$5:$A$24,A27))</f>
         <v/>
@@ -34368,14 +34639,42 @@
         <f>IF(OR(K27="",N(M27)&lt;=0),"",K27/M27)</f>
         <v/>
       </c>
-      <c r="S27" s="70" t="n"/>
+      <c r="S27" s="70" t="inlineStr">
+        <is>
+          <t>Por verificar en POT de Bello (Acuerdo vigente)</t>
+        </is>
+      </c>
       <c r="T27" s="70" t="n"/>
-      <c r="U27" s="70" t="n"/>
-      <c r="V27" s="70" t="n"/>
-      <c r="W27" s="70" t="n"/>
-      <c r="X27" s="70" t="n"/>
-      <c r="Y27" s="70" t="n"/>
-      <c r="Z27" s="74" t="n"/>
+      <c r="U27" s="70" t="inlineStr">
+        <is>
+          <t>Casa de 4 niveles, 4 alcobas, 3 baños, balcón; cada nivel 42 m², área total 168 m². Publicada hace 2 meses (a 05/10/2026). No publica régimen, administración ni coordenadas.</t>
+        </is>
+      </c>
+      <c r="V27" s="70" t="inlineStr">
+        <is>
+          <t>Aliadosinmobiliarios – MercadoLibre</t>
+        </is>
+      </c>
+      <c r="W27" s="70" t="inlineStr">
+        <is>
+          <t>Solicitar en portal</t>
+        </is>
+      </c>
+      <c r="X27" s="70" t="inlineStr">
+        <is>
+          <t>https://casa.mercadolibre.com.co/MCO-4221795790-se-vende-hermosa-casa-de-4-niveles-en-santa-ana-bello-de-168-mts-_JM</t>
+        </is>
+      </c>
+      <c r="Y27" s="70" t="inlineStr">
+        <is>
+          <t>Casa de 4 niveles, 168 m² construidos; incluida por decisión del perito. Falta régimen, administración y coordenadas.</t>
+        </is>
+      </c>
+      <c r="Z27" s="74" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="AA27" s="199">
         <f>IF(AND(Z27="SÍ",ISNUMBER(R27)),R27,"")</f>
         <v/>
@@ -35337,6 +35636,11 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X10" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X23" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X24" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X25" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X26" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="X27" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>